<commit_message>
removed ganz from spreadsheet
</commit_message>
<xml_diff>
--- a/party-comparison-updated-v78.xlsx
+++ b/party-comparison-updated-v78.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\einat\git_5050\party-comparison\party-comparison\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F02E1B88-050D-4697-B16E-50DB6BBE7ED0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDE4DB27-341E-4EE0-93BB-DD3854E47DEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-25125" yWindow="1485" windowWidth="21510" windowHeight="11295" tabRatio="500" firstSheet="5" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4305" yWindow="3615" windowWidth="21510" windowHeight="11295" tabRatio="500" firstSheet="5" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="כל הרשימות" sheetId="1" r:id="rId1"/>
@@ -120,7 +120,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7703" uniqueCount="1868">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7700" uniqueCount="1867">
   <si>
     <t>כלי תקשורת</t>
   </si>
@@ -5634,9 +5634,6 @@
   </si>
   <si>
     <t>מושב 6 (יאסר חוג'יראת) לא ודאי; יואב סגלוביץ' נוסף במיקום 2 לפי בקשת המשתמש (הצטרפות מיש עתיד/ביחד)</t>
-  </si>
-  <si>
-    <t>0 מנדטים חזויים (מתחת לסף שנקבע) - לא נספר</t>
   </si>
   <si>
     <t>מפלגה חדשה, הוקמה ע"י תא"ל (במיל') עופר וינטר; הושקה רשמית ב-25.8.2026. רשימה מבוססת דיווחי תקשורת ממסיבת ההשקה (ynet, ערוץ 7) - רשימה סופית וממוספרת רשמית טרם פורסמה לוועדת הבחירות המרכזית.</t>
@@ -44949,7 +44946,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -45005,7 +45002,7 @@
         <v>18</v>
       </c>
       <c r="E2">
-        <f t="shared" ref="E2:E17" si="0">IF(B2=0,0,C2/B2)</f>
+        <f t="shared" ref="E2:E16" si="0">IF(B2=0,0,C2/B2)</f>
         <v>0.14285714285714285</v>
       </c>
       <c r="F2" t="s">
@@ -45018,7 +45015,7 @@
         <v>7</v>
       </c>
       <c r="I2">
-        <f t="shared" ref="I2:I17" si="1">IF(G2=0,0,H2/G2)</f>
+        <f t="shared" ref="I2:I16" si="1">IF(G2=0,0,H2/G2)</f>
         <v>0.21875</v>
       </c>
     </row>
@@ -45364,7 +45361,7 @@
     </row>
     <row r="13" spans="1:9" ht="15" customHeight="1">
       <c r="A13" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="B13">
         <f>INDEX('סקר 2026'!$D:$D,MATCH(A13,'סקר 2026'!$A:$A,0))</f>
@@ -45386,35 +45383,35 @@
         <v>1838</v>
       </c>
       <c r="G13">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="H13">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I13">
         <f t="shared" si="1"/>
-        <v>0.25</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="15" customHeight="1">
       <c r="A14" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B14">
         <f>INDEX('סקר 2026'!$D:$D,MATCH(A14,'סקר 2026'!$A:$A,0))</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C14">
         <f>COUNTIFS('מועמדים 2026'!$A:$A,A14,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;B14)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D14">
         <f>COUNTIFS('מועמדים 2026'!$A:$A,A14,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;B14)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E14">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="F14" t="s">
         <v>1839</v>
@@ -45432,23 +45429,23 @@
     </row>
     <row r="15" spans="1:9" ht="15" customHeight="1">
       <c r="A15" t="s">
-        <v>23</v>
+        <v>1513</v>
       </c>
       <c r="B15">
         <f>INDEX('סקר 2026'!$D:$D,MATCH(A15,'סקר 2026'!$A:$A,0))</f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="C15">
         <f>COUNTIFS('מועמדים 2026'!$A:$A,A15,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;B15)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D15">
         <f>COUNTIFS('מועמדים 2026'!$A:$A,A15,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;B15)</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E15">
         <f t="shared" si="0"/>
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="F15" t="s">
         <v>1840</v>
@@ -45466,69 +45463,35 @@
     </row>
     <row r="16" spans="1:9" ht="15" customHeight="1">
       <c r="A16" t="s">
-        <v>1513</v>
+        <v>1841</v>
       </c>
       <c r="B16">
-        <f>INDEX('סקר 2026'!$D:$D,MATCH(A16,'סקר 2026'!$A:$A,0))</f>
-        <v>0</v>
+        <f>SUM(B2:B14)</f>
+        <v>119</v>
       </c>
       <c r="C16">
-        <f>COUNTIFS('מועמדים 2026'!$A:$A,A16,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;B16)</f>
-        <v>0</v>
+        <f>SUM(C2:C14)</f>
+        <v>32</v>
       </c>
       <c r="D16">
-        <f>COUNTIFS('מועמדים 2026'!$A:$A,A16,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;B16)</f>
-        <v>0</v>
+        <f>SUM(D2:D14)</f>
+        <v>87</v>
       </c>
       <c r="E16">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="F16" t="s">
-        <v>1841</v>
+        <v>0.26890756302521007</v>
       </c>
       <c r="G16">
-        <v>0</v>
+        <f>SUM(G2:G14)</f>
+        <v>107</v>
       </c>
       <c r="H16">
-        <v>0</v>
+        <f>SUM(H2:H14)</f>
+        <v>26</v>
       </c>
       <c r="I16">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" ht="15" customHeight="1">
-      <c r="A17" t="s">
-        <v>1842</v>
-      </c>
-      <c r="B17">
-        <f>SUM(B2:B15)</f>
-        <v>119</v>
-      </c>
-      <c r="C17">
-        <f>SUM(C2:C15)</f>
-        <v>32</v>
-      </c>
-      <c r="D17">
-        <f>SUM(D2:D15)</f>
-        <v>87</v>
-      </c>
-      <c r="E17">
-        <f t="shared" si="0"/>
-        <v>0.26890756302521007</v>
-      </c>
-      <c r="G17">
-        <f>SUM(G2:G15)</f>
-        <v>115</v>
-      </c>
-      <c r="H17">
-        <f>SUM(H2:H15)</f>
-        <v>28</v>
-      </c>
-      <c r="I17">
-        <f t="shared" si="1"/>
-        <v>0.24347826086956523</v>
+        <v>0.24299065420560748</v>
       </c>
     </row>
   </sheetData>
@@ -45540,10 +45503,10 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:S11"/>
+  <dimension ref="A1:R11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:19">
+    <row r="1" spans="1:18">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -45551,10 +45514,10 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
+        <v>1842</v>
+      </c>
+      <c r="D1" t="s">
         <v>1843</v>
-      </c>
-      <c r="D1" t="s">
-        <v>1844</v>
       </c>
       <c r="E1" t="s">
         <v>10</v>
@@ -45566,54 +45529,51 @@
         <v>12</v>
       </c>
       <c r="H1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="J1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="K1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="M1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="N1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="O1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="P1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="Q1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="R1" t="s">
-        <v>23</v>
-      </c>
-      <c r="S1" t="s">
         <v>1513</v>
       </c>
     </row>
-    <row r="2" spans="1:19">
+    <row r="2" spans="1:18">
       <c r="A2" t="s">
         <v>9</v>
       </c>
       <c r="B2" t="s">
+        <v>1844</v>
+      </c>
+      <c r="C2" t="s">
         <v>1845</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>1846</v>
-      </c>
-      <c r="D2" t="s">
-        <v>1847</v>
       </c>
       <c r="E2">
         <v>29</v>
@@ -45625,31 +45585,31 @@
         <v>10</v>
       </c>
       <c r="H2">
+        <v>7</v>
+      </c>
+      <c r="I2">
+        <v>6</v>
+      </c>
+      <c r="J2">
+        <v>8</v>
+      </c>
+      <c r="K2">
+        <v>7</v>
+      </c>
+      <c r="L2">
+        <v>6</v>
+      </c>
+      <c r="M2">
+        <v>7</v>
+      </c>
+      <c r="N2">
+        <v>10</v>
+      </c>
+      <c r="O2">
+        <v>22</v>
+      </c>
+      <c r="P2">
         <v>0</v>
-      </c>
-      <c r="I2">
-        <v>7</v>
-      </c>
-      <c r="J2">
-        <v>6</v>
-      </c>
-      <c r="K2">
-        <v>8</v>
-      </c>
-      <c r="L2">
-        <v>7</v>
-      </c>
-      <c r="M2">
-        <v>6</v>
-      </c>
-      <c r="N2">
-        <v>7</v>
-      </c>
-      <c r="O2">
-        <v>10</v>
-      </c>
-      <c r="P2">
-        <v>22</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -45657,22 +45617,19 @@
       <c r="R2">
         <v>0</v>
       </c>
-      <c r="S2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:19">
+    </row>
+    <row r="3" spans="1:18">
       <c r="A3" t="s">
         <v>24</v>
       </c>
       <c r="B3" t="s">
-        <v>1845</v>
+        <v>1844</v>
       </c>
       <c r="C3" t="s">
+        <v>1847</v>
+      </c>
+      <c r="D3" t="s">
         <v>1848</v>
-      </c>
-      <c r="D3" t="s">
-        <v>1849</v>
       </c>
       <c r="E3">
         <v>21</v>
@@ -45684,54 +45641,51 @@
         <v>8</v>
       </c>
       <c r="H3">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="I3">
         <v>8</v>
       </c>
       <c r="J3">
+        <v>9</v>
+      </c>
+      <c r="K3">
+        <v>7</v>
+      </c>
+      <c r="L3">
+        <v>5</v>
+      </c>
+      <c r="M3">
         <v>8</v>
       </c>
-      <c r="K3">
-        <v>9</v>
-      </c>
-      <c r="L3">
-        <v>7</v>
-      </c>
-      <c r="M3">
-        <v>5</v>
-      </c>
       <c r="N3">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="O3">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="P3">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="Q3">
+        <v>4</v>
+      </c>
+      <c r="R3">
         <v>0</v>
       </c>
-      <c r="R3">
-        <v>4</v>
-      </c>
-      <c r="S3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:19">
+    </row>
+    <row r="4" spans="1:18">
       <c r="A4" t="s">
         <v>25</v>
       </c>
       <c r="B4" t="s">
+        <v>1849</v>
+      </c>
+      <c r="C4" t="s">
         <v>1850</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>1851</v>
-      </c>
-      <c r="D4" t="s">
-        <v>1852</v>
       </c>
       <c r="E4">
         <v>18</v>
@@ -45743,54 +45697,51 @@
         <v>7</v>
       </c>
       <c r="H4">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="I4">
         <v>8</v>
       </c>
       <c r="J4">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K4">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="L4">
         <v>6</v>
       </c>
       <c r="M4">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="N4">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="O4">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="P4">
-        <v>21</v>
+        <v>4</v>
       </c>
       <c r="Q4">
         <v>4</v>
       </c>
       <c r="R4">
-        <v>4</v>
-      </c>
-      <c r="S4">
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:19">
+    <row r="5" spans="1:18">
       <c r="A5" t="s">
         <v>26</v>
       </c>
       <c r="B5" t="s">
+        <v>1852</v>
+      </c>
+      <c r="C5" t="s">
+        <v>1847</v>
+      </c>
+      <c r="D5" t="s">
         <v>1853</v>
-      </c>
-      <c r="C5" t="s">
-        <v>1848</v>
-      </c>
-      <c r="D5" t="s">
-        <v>1854</v>
       </c>
       <c r="E5">
         <v>21</v>
@@ -45802,54 +45753,51 @@
         <v>7</v>
       </c>
       <c r="H5">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="I5">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J5">
         <v>8</v>
       </c>
       <c r="K5">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="L5">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M5">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="N5">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="O5">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="P5">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="Q5">
+        <v>4</v>
+      </c>
+      <c r="R5">
         <v>0</v>
       </c>
-      <c r="R5">
-        <v>4</v>
-      </c>
-      <c r="S5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:19">
+    </row>
+    <row r="6" spans="1:18">
       <c r="A6" t="s">
         <v>27</v>
       </c>
       <c r="B6" t="s">
-        <v>1853</v>
+        <v>1852</v>
       </c>
       <c r="C6" t="s">
+        <v>1854</v>
+      </c>
+      <c r="D6" t="s">
         <v>1855</v>
-      </c>
-      <c r="D6" t="s">
-        <v>1856</v>
       </c>
       <c r="E6">
         <v>20</v>
@@ -45861,54 +45809,51 @@
         <v>8</v>
       </c>
       <c r="H6">
+        <v>8</v>
+      </c>
+      <c r="I6">
+        <v>9</v>
+      </c>
+      <c r="J6">
+        <v>8</v>
+      </c>
+      <c r="K6">
+        <v>6</v>
+      </c>
+      <c r="L6">
+        <v>5</v>
+      </c>
+      <c r="M6">
+        <v>7</v>
+      </c>
+      <c r="N6">
+        <v>11</v>
+      </c>
+      <c r="O6">
+        <v>26</v>
+      </c>
+      <c r="P6">
         <v>0</v>
       </c>
-      <c r="I6">
-        <v>8</v>
-      </c>
-      <c r="J6">
-        <v>9</v>
-      </c>
-      <c r="K6">
-        <v>8</v>
-      </c>
-      <c r="L6">
-        <v>6</v>
-      </c>
-      <c r="M6">
-        <v>5</v>
-      </c>
-      <c r="N6">
-        <v>7</v>
-      </c>
-      <c r="O6">
-        <v>11</v>
-      </c>
-      <c r="P6">
-        <v>26</v>
-      </c>
       <c r="Q6">
+        <v>4</v>
+      </c>
+      <c r="R6">
         <v>0</v>
       </c>
-      <c r="R6">
-        <v>4</v>
-      </c>
-      <c r="S6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:19">
+    </row>
+    <row r="7" spans="1:18">
       <c r="A7" t="s">
         <v>28</v>
       </c>
       <c r="B7" t="s">
+        <v>1856</v>
+      </c>
+      <c r="C7" t="s">
         <v>1857</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>1858</v>
-      </c>
-      <c r="D7" t="s">
-        <v>1859</v>
       </c>
       <c r="E7">
         <v>18</v>
@@ -45920,7 +45865,7 @@
         <v>7</v>
       </c>
       <c r="H7">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="I7">
         <v>9</v>
@@ -45929,45 +45874,42 @@
         <v>9</v>
       </c>
       <c r="K7">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="L7">
         <v>6</v>
       </c>
       <c r="M7">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="N7">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="O7">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="P7">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="Q7">
         <v>4</v>
       </c>
       <c r="R7">
-        <v>4</v>
-      </c>
-      <c r="S7">
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:19">
+    <row r="8" spans="1:18">
       <c r="A8" t="s">
         <v>29</v>
       </c>
       <c r="B8" t="s">
+        <v>1859</v>
+      </c>
+      <c r="C8" t="s">
         <v>1860</v>
       </c>
-      <c r="C8" t="s">
-        <v>1861</v>
-      </c>
       <c r="D8" t="s">
-        <v>1856</v>
+        <v>1855</v>
       </c>
       <c r="E8">
         <v>18</v>
@@ -45979,54 +45921,51 @@
         <v>7</v>
       </c>
       <c r="H8">
+        <v>8</v>
+      </c>
+      <c r="I8">
+        <v>7</v>
+      </c>
+      <c r="J8">
+        <v>9</v>
+      </c>
+      <c r="K8">
+        <v>6</v>
+      </c>
+      <c r="L8">
+        <v>5</v>
+      </c>
+      <c r="M8">
+        <v>9</v>
+      </c>
+      <c r="N8">
+        <v>13</v>
+      </c>
+      <c r="O8">
+        <v>21</v>
+      </c>
+      <c r="P8">
+        <v>4</v>
+      </c>
+      <c r="Q8">
+        <v>5</v>
+      </c>
+      <c r="R8">
         <v>0</v>
       </c>
-      <c r="I8">
-        <v>8</v>
-      </c>
-      <c r="J8">
-        <v>7</v>
-      </c>
-      <c r="K8">
-        <v>9</v>
-      </c>
-      <c r="L8">
-        <v>6</v>
-      </c>
-      <c r="M8">
-        <v>5</v>
-      </c>
-      <c r="N8">
-        <v>9</v>
-      </c>
-      <c r="O8">
-        <v>13</v>
-      </c>
-      <c r="P8">
-        <v>21</v>
-      </c>
-      <c r="Q8">
-        <v>4</v>
-      </c>
-      <c r="R8">
-        <v>5</v>
-      </c>
-      <c r="S8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:19">
+    </row>
+    <row r="9" spans="1:18">
       <c r="A9" t="s">
         <v>30</v>
       </c>
       <c r="B9" t="s">
+        <v>1861</v>
+      </c>
+      <c r="C9" t="s">
         <v>1862</v>
       </c>
-      <c r="C9" t="s">
+      <c r="D9" t="s">
         <v>1863</v>
-      </c>
-      <c r="D9" t="s">
-        <v>1864</v>
       </c>
       <c r="E9">
         <v>20</v>
@@ -46038,54 +45977,51 @@
         <v>8</v>
       </c>
       <c r="H9">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="I9">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J9">
         <v>9</v>
       </c>
       <c r="K9">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="L9">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M9">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="N9">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="O9">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="P9">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="Q9">
+        <v>4</v>
+      </c>
+      <c r="R9">
         <v>0</v>
       </c>
-      <c r="R9">
-        <v>4</v>
-      </c>
-      <c r="S9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:19">
+    </row>
+    <row r="10" spans="1:18">
       <c r="A10" t="s">
         <v>31</v>
       </c>
       <c r="B10" t="s">
-        <v>1862</v>
+        <v>1861</v>
       </c>
       <c r="C10" t="s">
-        <v>1851</v>
+        <v>1850</v>
       </c>
       <c r="D10" t="s">
-        <v>1856</v>
+        <v>1855</v>
       </c>
       <c r="E10">
         <v>20</v>
@@ -46097,54 +46033,51 @@
         <v>7</v>
       </c>
       <c r="H10">
+        <v>8</v>
+      </c>
+      <c r="I10">
+        <v>9</v>
+      </c>
+      <c r="J10">
+        <v>10</v>
+      </c>
+      <c r="K10">
+        <v>6</v>
+      </c>
+      <c r="L10">
+        <v>5</v>
+      </c>
+      <c r="M10">
+        <v>8</v>
+      </c>
+      <c r="N10">
+        <v>13</v>
+      </c>
+      <c r="O10">
+        <v>22</v>
+      </c>
+      <c r="P10">
         <v>0</v>
       </c>
-      <c r="I10">
-        <v>8</v>
-      </c>
-      <c r="J10">
-        <v>9</v>
-      </c>
-      <c r="K10">
-        <v>10</v>
-      </c>
-      <c r="L10">
-        <v>6</v>
-      </c>
-      <c r="M10">
-        <v>5</v>
-      </c>
-      <c r="N10">
-        <v>8</v>
-      </c>
-      <c r="O10">
-        <v>13</v>
-      </c>
-      <c r="P10">
-        <v>22</v>
-      </c>
       <c r="Q10">
+        <v>4</v>
+      </c>
+      <c r="R10">
         <v>0</v>
       </c>
-      <c r="R10">
-        <v>4</v>
-      </c>
-      <c r="S10">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:19">
+    </row>
+    <row r="11" spans="1:18">
       <c r="A11" t="s">
         <v>32</v>
       </c>
       <c r="B11" t="s">
+        <v>1864</v>
+      </c>
+      <c r="C11" t="s">
         <v>1865</v>
       </c>
-      <c r="C11" t="s">
+      <c r="D11" t="s">
         <v>1866</v>
-      </c>
-      <c r="D11" t="s">
-        <v>1867</v>
       </c>
       <c r="E11">
         <v>26</v>
@@ -46156,39 +46089,36 @@
         <v>7</v>
       </c>
       <c r="H11">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="I11">
         <v>7</v>
       </c>
       <c r="J11">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="K11">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="L11">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M11">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="N11">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="O11">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="P11">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="Q11">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="R11">
-        <v>0</v>
-      </c>
-      <c r="S11">
         <v>0</v>
       </c>
     </row>
@@ -46350,9 +46280,9 @@
       <c r="C5" t="s">
         <v>13</v>
       </c>
-      <c r="D5">
-        <f>INDEX('סקרים לפי ערוץ'!H:H,MATCH($A5,'סקרים לפי ערוץ'!$A:$A,0))</f>
-        <v>0</v>
+      <c r="D5" t="e">
+        <f>INDEX('סקרים לפי ערוץ'!#REF!,MATCH($A5,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>#REF!</v>
       </c>
       <c r="E5">
         <f>COUNTIFS('מועמדים 2026'!$A:$A,$C5,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D5)</f>
@@ -46362,17 +46292,17 @@
         <f>COUNTIFS('מועמדים 2026'!$A:$A,$C5,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D5)</f>
         <v>0</v>
       </c>
-      <c r="G5">
+      <c r="G5" t="e">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>#REF!</v>
       </c>
       <c r="H5">
         <f>COUNTIFS('מועמדים 2026'!$A:$A,$C5)</f>
         <v>5</v>
       </c>
-      <c r="I5" t="str">
+      <c r="I5" t="e">
         <f t="shared" si="1"/>
-        <v/>
+        <v>#REF!</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -46387,7 +46317,7 @@
         <v>14</v>
       </c>
       <c r="D6">
-        <f>INDEX('סקרים לפי ערוץ'!I:I,MATCH($A6,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!H:H,MATCH($A6,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>7</v>
       </c>
       <c r="E6">
@@ -46423,7 +46353,7 @@
         <v>15</v>
       </c>
       <c r="D7">
-        <f>INDEX('סקרים לפי ערוץ'!J:J,MATCH($A7,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!I:I,MATCH($A7,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>6</v>
       </c>
       <c r="E7">
@@ -46459,7 +46389,7 @@
         <v>16</v>
       </c>
       <c r="D8">
-        <f>INDEX('סקרים לפי ערוץ'!K:K,MATCH($A8,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!J:J,MATCH($A8,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>8</v>
       </c>
       <c r="E8">
@@ -46495,7 +46425,7 @@
         <v>17</v>
       </c>
       <c r="D9">
-        <f>INDEX('סקרים לפי ערוץ'!L:L,MATCH($A9,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!K:K,MATCH($A9,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>7</v>
       </c>
       <c r="E9">
@@ -46531,7 +46461,7 @@
         <v>18</v>
       </c>
       <c r="D10">
-        <f>INDEX('סקרים לפי ערוץ'!M:M,MATCH($A10,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!L:L,MATCH($A10,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>6</v>
       </c>
       <c r="E10">
@@ -46567,7 +46497,7 @@
         <v>19</v>
       </c>
       <c r="D11">
-        <f>INDEX('סקרים לפי ערוץ'!N:N,MATCH($A11,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!M:M,MATCH($A11,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>7</v>
       </c>
       <c r="E11">
@@ -46603,7 +46533,7 @@
         <v>20</v>
       </c>
       <c r="D12">
-        <f>INDEX('סקרים לפי ערוץ'!O:O,MATCH($A12,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!N:N,MATCH($A12,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>10</v>
       </c>
       <c r="E12">
@@ -46639,7 +46569,7 @@
         <v>21</v>
       </c>
       <c r="D13">
-        <f>INDEX('סקרים לפי ערוץ'!P:P,MATCH($A13,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!O:O,MATCH($A13,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>22</v>
       </c>
       <c r="E13">
@@ -46675,7 +46605,7 @@
         <v>22</v>
       </c>
       <c r="D14">
-        <f>INDEX('סקרים לפי ערוץ'!Q:Q,MATCH($A14,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!P:P,MATCH($A14,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>0</v>
       </c>
       <c r="E14">
@@ -46711,7 +46641,7 @@
         <v>23</v>
       </c>
       <c r="D15">
-        <f>INDEX('סקרים לפי ערוץ'!R:R,MATCH($A15,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!Q:Q,MATCH($A15,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>0</v>
       </c>
       <c r="E15">
@@ -46854,9 +46784,9 @@
       <c r="C19" t="s">
         <v>13</v>
       </c>
-      <c r="D19">
-        <f>INDEX('סקרים לפי ערוץ'!H:H,MATCH($A19,'סקרים לפי ערוץ'!$A:$A,0))</f>
-        <v>0</v>
+      <c r="D19" t="e">
+        <f>INDEX('סקרים לפי ערוץ'!#REF!,MATCH($A19,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>#REF!</v>
       </c>
       <c r="E19">
         <f>COUNTIFS('מועמדים 2026'!$A:$A,$C19,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D19)</f>
@@ -46866,17 +46796,17 @@
         <f>COUNTIFS('מועמדים 2026'!$A:$A,$C19,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D19)</f>
         <v>0</v>
       </c>
-      <c r="G19">
+      <c r="G19" t="e">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>#REF!</v>
       </c>
       <c r="H19">
         <f>COUNTIFS('מועמדים 2026'!$A:$A,$C19)</f>
         <v>5</v>
       </c>
-      <c r="I19" t="str">
+      <c r="I19" t="e">
         <f t="shared" si="1"/>
-        <v/>
+        <v>#REF!</v>
       </c>
     </row>
     <row r="20" spans="1:9">
@@ -46891,7 +46821,7 @@
         <v>14</v>
       </c>
       <c r="D20">
-        <f>INDEX('סקרים לפי ערוץ'!I:I,MATCH($A20,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!H:H,MATCH($A20,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>8</v>
       </c>
       <c r="E20">
@@ -46927,7 +46857,7 @@
         <v>15</v>
       </c>
       <c r="D21">
-        <f>INDEX('סקרים לפי ערוץ'!J:J,MATCH($A21,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!I:I,MATCH($A21,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>8</v>
       </c>
       <c r="E21">
@@ -46963,7 +46893,7 @@
         <v>16</v>
       </c>
       <c r="D22">
-        <f>INDEX('סקרים לפי ערוץ'!K:K,MATCH($A22,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!J:J,MATCH($A22,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>9</v>
       </c>
       <c r="E22">
@@ -46999,7 +46929,7 @@
         <v>17</v>
       </c>
       <c r="D23">
-        <f>INDEX('סקרים לפי ערוץ'!L:L,MATCH($A23,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!K:K,MATCH($A23,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>7</v>
       </c>
       <c r="E23">
@@ -47035,7 +46965,7 @@
         <v>18</v>
       </c>
       <c r="D24">
-        <f>INDEX('סקרים לפי ערוץ'!M:M,MATCH($A24,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!L:L,MATCH($A24,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>5</v>
       </c>
       <c r="E24">
@@ -47071,7 +47001,7 @@
         <v>19</v>
       </c>
       <c r="D25">
-        <f>INDEX('סקרים לפי ערוץ'!N:N,MATCH($A25,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!M:M,MATCH($A25,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>8</v>
       </c>
       <c r="E25">
@@ -47107,7 +47037,7 @@
         <v>20</v>
       </c>
       <c r="D26">
-        <f>INDEX('סקרים לפי ערוץ'!O:O,MATCH($A26,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!N:N,MATCH($A26,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>12</v>
       </c>
       <c r="E26">
@@ -47143,7 +47073,7 @@
         <v>21</v>
       </c>
       <c r="D27">
-        <f>INDEX('סקרים לפי ערוץ'!P:P,MATCH($A27,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!O:O,MATCH($A27,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>23</v>
       </c>
       <c r="E27">
@@ -47179,7 +47109,7 @@
         <v>22</v>
       </c>
       <c r="D28">
-        <f>INDEX('סקרים לפי ערוץ'!Q:Q,MATCH($A28,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!P:P,MATCH($A28,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>0</v>
       </c>
       <c r="E28">
@@ -47215,7 +47145,7 @@
         <v>23</v>
       </c>
       <c r="D29">
-        <f>INDEX('סקרים לפי ערוץ'!R:R,MATCH($A29,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!Q:Q,MATCH($A29,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>4</v>
       </c>
       <c r="E29">
@@ -47358,9 +47288,9 @@
       <c r="C33" t="s">
         <v>13</v>
       </c>
-      <c r="D33">
-        <f>INDEX('סקרים לפי ערוץ'!H:H,MATCH($A33,'סקרים לפי ערוץ'!$A:$A,0))</f>
-        <v>0</v>
+      <c r="D33" t="e">
+        <f>INDEX('סקרים לפי ערוץ'!#REF!,MATCH($A33,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>#REF!</v>
       </c>
       <c r="E33">
         <f>COUNTIFS('מועמדים 2026'!$A:$A,$C33,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D33)</f>
@@ -47370,17 +47300,17 @@
         <f>COUNTIFS('מועמדים 2026'!$A:$A,$C33,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D33)</f>
         <v>0</v>
       </c>
-      <c r="G33">
+      <c r="G33" t="e">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>#REF!</v>
       </c>
       <c r="H33">
         <f>COUNTIFS('מועמדים 2026'!$A:$A,$C33)</f>
         <v>5</v>
       </c>
-      <c r="I33" t="str">
+      <c r="I33" t="e">
         <f t="shared" si="1"/>
-        <v/>
+        <v>#REF!</v>
       </c>
     </row>
     <row r="34" spans="1:9">
@@ -47395,7 +47325,7 @@
         <v>14</v>
       </c>
       <c r="D34">
-        <f>INDEX('סקרים לפי ערוץ'!I:I,MATCH($A34,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!H:H,MATCH($A34,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>8</v>
       </c>
       <c r="E34">
@@ -47431,7 +47361,7 @@
         <v>15</v>
       </c>
       <c r="D35">
-        <f>INDEX('סקרים לפי ערוץ'!J:J,MATCH($A35,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!I:I,MATCH($A35,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>8</v>
       </c>
       <c r="E35">
@@ -47467,7 +47397,7 @@
         <v>16</v>
       </c>
       <c r="D36">
-        <f>INDEX('סקרים לפי ערוץ'!K:K,MATCH($A36,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!J:J,MATCH($A36,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>9</v>
       </c>
       <c r="E36">
@@ -47503,7 +47433,7 @@
         <v>17</v>
       </c>
       <c r="D37">
-        <f>INDEX('סקרים לפי ערוץ'!L:L,MATCH($A37,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!K:K,MATCH($A37,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>6</v>
       </c>
       <c r="E37">
@@ -47539,7 +47469,7 @@
         <v>18</v>
       </c>
       <c r="D38">
-        <f>INDEX('סקרים לפי ערוץ'!M:M,MATCH($A38,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!L:L,MATCH($A38,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>6</v>
       </c>
       <c r="E38">
@@ -47575,7 +47505,7 @@
         <v>19</v>
       </c>
       <c r="D39">
-        <f>INDEX('סקרים לפי ערוץ'!N:N,MATCH($A39,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!M:M,MATCH($A39,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>8</v>
       </c>
       <c r="E39">
@@ -47611,7 +47541,7 @@
         <v>20</v>
       </c>
       <c r="D40">
-        <f>INDEX('סקרים לפי ערוץ'!O:O,MATCH($A40,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!N:N,MATCH($A40,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>13</v>
       </c>
       <c r="E40">
@@ -47647,7 +47577,7 @@
         <v>21</v>
       </c>
       <c r="D41">
-        <f>INDEX('סקרים לפי ערוץ'!P:P,MATCH($A41,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!O:O,MATCH($A41,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>21</v>
       </c>
       <c r="E41">
@@ -47683,7 +47613,7 @@
         <v>22</v>
       </c>
       <c r="D42">
-        <f>INDEX('סקרים לפי ערוץ'!Q:Q,MATCH($A42,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!P:P,MATCH($A42,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>4</v>
       </c>
       <c r="E42">
@@ -47719,7 +47649,7 @@
         <v>23</v>
       </c>
       <c r="D43">
-        <f>INDEX('סקרים לפי ערוץ'!R:R,MATCH($A43,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!Q:Q,MATCH($A43,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>4</v>
       </c>
       <c r="E43">
@@ -47862,9 +47792,9 @@
       <c r="C47" t="s">
         <v>13</v>
       </c>
-      <c r="D47">
-        <f>INDEX('סקרים לפי ערוץ'!H:H,MATCH($A47,'סקרים לפי ערוץ'!$A:$A,0))</f>
-        <v>0</v>
+      <c r="D47" t="e">
+        <f>INDEX('סקרים לפי ערוץ'!#REF!,MATCH($A47,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>#REF!</v>
       </c>
       <c r="E47">
         <f>COUNTIFS('מועמדים 2026'!$A:$A,$C47,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D47)</f>
@@ -47874,17 +47804,17 @@
         <f>COUNTIFS('מועמדים 2026'!$A:$A,$C47,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D47)</f>
         <v>0</v>
       </c>
-      <c r="G47">
+      <c r="G47" t="e">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>#REF!</v>
       </c>
       <c r="H47">
         <f>COUNTIFS('מועמדים 2026'!$A:$A,$C47)</f>
         <v>5</v>
       </c>
-      <c r="I47" t="str">
+      <c r="I47" t="e">
         <f t="shared" si="1"/>
-        <v/>
+        <v>#REF!</v>
       </c>
     </row>
     <row r="48" spans="1:9">
@@ -47899,7 +47829,7 @@
         <v>14</v>
       </c>
       <c r="D48">
-        <f>INDEX('סקרים לפי ערוץ'!I:I,MATCH($A48,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!H:H,MATCH($A48,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>9</v>
       </c>
       <c r="E48">
@@ -47935,7 +47865,7 @@
         <v>15</v>
       </c>
       <c r="D49">
-        <f>INDEX('סקרים לפי ערוץ'!J:J,MATCH($A49,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!I:I,MATCH($A49,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>8</v>
       </c>
       <c r="E49">
@@ -47971,7 +47901,7 @@
         <v>16</v>
       </c>
       <c r="D50">
-        <f>INDEX('סקרים לפי ערוץ'!K:K,MATCH($A50,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!J:J,MATCH($A50,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>8</v>
       </c>
       <c r="E50">
@@ -48007,7 +47937,7 @@
         <v>17</v>
       </c>
       <c r="D51">
-        <f>INDEX('סקרים לפי ערוץ'!L:L,MATCH($A51,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!K:K,MATCH($A51,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>6</v>
       </c>
       <c r="E51">
@@ -48043,7 +47973,7 @@
         <v>18</v>
       </c>
       <c r="D52">
-        <f>INDEX('סקרים לפי ערוץ'!M:M,MATCH($A52,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!L:L,MATCH($A52,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>5</v>
       </c>
       <c r="E52">
@@ -48079,7 +48009,7 @@
         <v>19</v>
       </c>
       <c r="D53">
-        <f>INDEX('סקרים לפי ערוץ'!N:N,MATCH($A53,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!M:M,MATCH($A53,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>9</v>
       </c>
       <c r="E53">
@@ -48115,7 +48045,7 @@
         <v>20</v>
       </c>
       <c r="D54">
-        <f>INDEX('סקרים לפי ערוץ'!O:O,MATCH($A54,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!N:N,MATCH($A54,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>12</v>
       </c>
       <c r="E54">
@@ -48151,7 +48081,7 @@
         <v>21</v>
       </c>
       <c r="D55">
-        <f>INDEX('סקרים לפי ערוץ'!P:P,MATCH($A55,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!O:O,MATCH($A55,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>24</v>
       </c>
       <c r="E55">
@@ -48187,7 +48117,7 @@
         <v>22</v>
       </c>
       <c r="D56">
-        <f>INDEX('סקרים לפי ערוץ'!Q:Q,MATCH($A56,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!P:P,MATCH($A56,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>0</v>
       </c>
       <c r="E56">
@@ -48223,7 +48153,7 @@
         <v>23</v>
       </c>
       <c r="D57">
-        <f>INDEX('סקרים לפי ערוץ'!R:R,MATCH($A57,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!Q:Q,MATCH($A57,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>4</v>
       </c>
       <c r="E57">
@@ -48366,9 +48296,9 @@
       <c r="C61" t="s">
         <v>13</v>
       </c>
-      <c r="D61">
-        <f>INDEX('סקרים לפי ערוץ'!H:H,MATCH($A61,'סקרים לפי ערוץ'!$A:$A,0))</f>
-        <v>0</v>
+      <c r="D61" t="e">
+        <f>INDEX('סקרים לפי ערוץ'!#REF!,MATCH($A61,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>#REF!</v>
       </c>
       <c r="E61">
         <f>COUNTIFS('מועמדים 2026'!$A:$A,$C61,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D61)</f>
@@ -48378,17 +48308,17 @@
         <f>COUNTIFS('מועמדים 2026'!$A:$A,$C61,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D61)</f>
         <v>0</v>
       </c>
-      <c r="G61">
+      <c r="G61" t="e">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>#REF!</v>
       </c>
       <c r="H61">
         <f>COUNTIFS('מועמדים 2026'!$A:$A,$C61)</f>
         <v>5</v>
       </c>
-      <c r="I61" t="str">
+      <c r="I61" t="e">
         <f t="shared" si="1"/>
-        <v/>
+        <v>#REF!</v>
       </c>
     </row>
     <row r="62" spans="1:9">
@@ -48403,7 +48333,7 @@
         <v>14</v>
       </c>
       <c r="D62">
-        <f>INDEX('סקרים לפי ערוץ'!I:I,MATCH($A62,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!H:H,MATCH($A62,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>8</v>
       </c>
       <c r="E62">
@@ -48439,7 +48369,7 @@
         <v>15</v>
       </c>
       <c r="D63">
-        <f>INDEX('סקרים לפי ערוץ'!J:J,MATCH($A63,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!I:I,MATCH($A63,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>9</v>
       </c>
       <c r="E63">
@@ -48475,7 +48405,7 @@
         <v>16</v>
       </c>
       <c r="D64">
-        <f>INDEX('סקרים לפי ערוץ'!K:K,MATCH($A64,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!J:J,MATCH($A64,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>8</v>
       </c>
       <c r="E64">
@@ -48511,7 +48441,7 @@
         <v>17</v>
       </c>
       <c r="D65">
-        <f>INDEX('סקרים לפי ערוץ'!L:L,MATCH($A65,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!K:K,MATCH($A65,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>6</v>
       </c>
       <c r="E65">
@@ -48547,7 +48477,7 @@
         <v>18</v>
       </c>
       <c r="D66">
-        <f>INDEX('סקרים לפי ערוץ'!M:M,MATCH($A66,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!L:L,MATCH($A66,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>5</v>
       </c>
       <c r="E66">
@@ -48583,7 +48513,7 @@
         <v>19</v>
       </c>
       <c r="D67">
-        <f>INDEX('סקרים לפי ערוץ'!N:N,MATCH($A67,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!M:M,MATCH($A67,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>7</v>
       </c>
       <c r="E67">
@@ -48619,7 +48549,7 @@
         <v>20</v>
       </c>
       <c r="D68">
-        <f>INDEX('סקרים לפי ערוץ'!O:O,MATCH($A68,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!N:N,MATCH($A68,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>11</v>
       </c>
       <c r="E68">
@@ -48655,7 +48585,7 @@
         <v>21</v>
       </c>
       <c r="D69">
-        <f>INDEX('סקרים לפי ערוץ'!P:P,MATCH($A69,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!O:O,MATCH($A69,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>26</v>
       </c>
       <c r="E69">
@@ -48691,7 +48621,7 @@
         <v>22</v>
       </c>
       <c r="D70">
-        <f>INDEX('סקרים לפי ערוץ'!Q:Q,MATCH($A70,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!P:P,MATCH($A70,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>0</v>
       </c>
       <c r="E70">
@@ -48727,7 +48657,7 @@
         <v>23</v>
       </c>
       <c r="D71">
-        <f>INDEX('סקרים לפי ערוץ'!R:R,MATCH($A71,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!Q:Q,MATCH($A71,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>4</v>
       </c>
       <c r="E71">
@@ -48870,9 +48800,9 @@
       <c r="C75" t="s">
         <v>13</v>
       </c>
-      <c r="D75">
-        <f>INDEX('סקרים לפי ערוץ'!H:H,MATCH($A75,'סקרים לפי ערוץ'!$A:$A,0))</f>
-        <v>0</v>
+      <c r="D75" t="e">
+        <f>INDEX('סקרים לפי ערוץ'!#REF!,MATCH($A75,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>#REF!</v>
       </c>
       <c r="E75">
         <f>COUNTIFS('מועמדים 2026'!$A:$A,$C75,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D75)</f>
@@ -48882,17 +48812,17 @@
         <f>COUNTIFS('מועמדים 2026'!$A:$A,$C75,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D75)</f>
         <v>0</v>
       </c>
-      <c r="G75">
+      <c r="G75" t="e">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>#REF!</v>
       </c>
       <c r="H75">
         <f>COUNTIFS('מועמדים 2026'!$A:$A,$C75)</f>
         <v>5</v>
       </c>
-      <c r="I75" t="str">
+      <c r="I75" t="e">
         <f t="shared" si="4"/>
-        <v/>
+        <v>#REF!</v>
       </c>
     </row>
     <row r="76" spans="1:9">
@@ -48907,7 +48837,7 @@
         <v>14</v>
       </c>
       <c r="D76">
-        <f>INDEX('סקרים לפי ערוץ'!I:I,MATCH($A76,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!H:H,MATCH($A76,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>9</v>
       </c>
       <c r="E76">
@@ -48943,7 +48873,7 @@
         <v>15</v>
       </c>
       <c r="D77">
-        <f>INDEX('סקרים לפי ערוץ'!J:J,MATCH($A77,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!I:I,MATCH($A77,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>9</v>
       </c>
       <c r="E77">
@@ -48979,7 +48909,7 @@
         <v>16</v>
       </c>
       <c r="D78">
-        <f>INDEX('סקרים לפי ערוץ'!K:K,MATCH($A78,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!J:J,MATCH($A78,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>9</v>
       </c>
       <c r="E78">
@@ -49015,7 +48945,7 @@
         <v>17</v>
       </c>
       <c r="D79">
-        <f>INDEX('סקרים לפי ערוץ'!L:L,MATCH($A79,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!K:K,MATCH($A79,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>6</v>
       </c>
       <c r="E79">
@@ -49051,7 +48981,7 @@
         <v>18</v>
       </c>
       <c r="D80">
-        <f>INDEX('סקרים לפי ערוץ'!M:M,MATCH($A80,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!L:L,MATCH($A80,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>6</v>
       </c>
       <c r="E80">
@@ -49087,7 +49017,7 @@
         <v>19</v>
       </c>
       <c r="D81">
-        <f>INDEX('סקרים לפי ערוץ'!N:N,MATCH($A81,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!M:M,MATCH($A81,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>8</v>
       </c>
       <c r="E81">
@@ -49123,7 +49053,7 @@
         <v>20</v>
       </c>
       <c r="D82">
-        <f>INDEX('סקרים לפי ערוץ'!O:O,MATCH($A82,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!N:N,MATCH($A82,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>12</v>
       </c>
       <c r="E82">
@@ -49159,7 +49089,7 @@
         <v>21</v>
       </c>
       <c r="D83">
-        <f>INDEX('סקרים לפי ערוץ'!P:P,MATCH($A83,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!O:O,MATCH($A83,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>20</v>
       </c>
       <c r="E83">
@@ -49195,7 +49125,7 @@
         <v>22</v>
       </c>
       <c r="D84">
-        <f>INDEX('סקרים לפי ערוץ'!Q:Q,MATCH($A84,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!P:P,MATCH($A84,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>4</v>
       </c>
       <c r="E84">
@@ -49231,7 +49161,7 @@
         <v>23</v>
       </c>
       <c r="D85">
-        <f>INDEX('סקרים לפי ערוץ'!R:R,MATCH($A85,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!Q:Q,MATCH($A85,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>4</v>
       </c>
       <c r="E85">
@@ -49374,9 +49304,9 @@
       <c r="C89" t="s">
         <v>13</v>
       </c>
-      <c r="D89">
-        <f>INDEX('סקרים לפי ערוץ'!H:H,MATCH($A89,'סקרים לפי ערוץ'!$A:$A,0))</f>
-        <v>0</v>
+      <c r="D89" t="e">
+        <f>INDEX('סקרים לפי ערוץ'!#REF!,MATCH($A89,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>#REF!</v>
       </c>
       <c r="E89">
         <f>COUNTIFS('מועמדים 2026'!$A:$A,$C89,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D89)</f>
@@ -49386,17 +49316,17 @@
         <f>COUNTIFS('מועמדים 2026'!$A:$A,$C89,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D89)</f>
         <v>0</v>
       </c>
-      <c r="G89">
+      <c r="G89" t="e">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>#REF!</v>
       </c>
       <c r="H89">
         <f>COUNTIFS('מועמדים 2026'!$A:$A,$C89)</f>
         <v>5</v>
       </c>
-      <c r="I89" t="str">
+      <c r="I89" t="e">
         <f t="shared" si="4"/>
-        <v/>
+        <v>#REF!</v>
       </c>
     </row>
     <row r="90" spans="1:9">
@@ -49411,7 +49341,7 @@
         <v>14</v>
       </c>
       <c r="D90">
-        <f>INDEX('סקרים לפי ערוץ'!I:I,MATCH($A90,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!H:H,MATCH($A90,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>8</v>
       </c>
       <c r="E90">
@@ -49447,7 +49377,7 @@
         <v>15</v>
       </c>
       <c r="D91">
-        <f>INDEX('סקרים לפי ערוץ'!J:J,MATCH($A91,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!I:I,MATCH($A91,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>7</v>
       </c>
       <c r="E91">
@@ -49483,7 +49413,7 @@
         <v>16</v>
       </c>
       <c r="D92">
-        <f>INDEX('סקרים לפי ערוץ'!K:K,MATCH($A92,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!J:J,MATCH($A92,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>9</v>
       </c>
       <c r="E92">
@@ -49519,7 +49449,7 @@
         <v>17</v>
       </c>
       <c r="D93">
-        <f>INDEX('סקרים לפי ערוץ'!L:L,MATCH($A93,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!K:K,MATCH($A93,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>6</v>
       </c>
       <c r="E93">
@@ -49555,7 +49485,7 @@
         <v>18</v>
       </c>
       <c r="D94">
-        <f>INDEX('סקרים לפי ערוץ'!M:M,MATCH($A94,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!L:L,MATCH($A94,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>5</v>
       </c>
       <c r="E94">
@@ -49591,7 +49521,7 @@
         <v>19</v>
       </c>
       <c r="D95">
-        <f>INDEX('סקרים לפי ערוץ'!N:N,MATCH($A95,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!M:M,MATCH($A95,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>9</v>
       </c>
       <c r="E95">
@@ -49627,7 +49557,7 @@
         <v>20</v>
       </c>
       <c r="D96">
-        <f>INDEX('סקרים לפי ערוץ'!O:O,MATCH($A96,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!N:N,MATCH($A96,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>13</v>
       </c>
       <c r="E96">
@@ -49663,7 +49593,7 @@
         <v>21</v>
       </c>
       <c r="D97">
-        <f>INDEX('סקרים לפי ערוץ'!P:P,MATCH($A97,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!O:O,MATCH($A97,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>21</v>
       </c>
       <c r="E97">
@@ -49699,7 +49629,7 @@
         <v>22</v>
       </c>
       <c r="D98">
-        <f>INDEX('סקרים לפי ערוץ'!Q:Q,MATCH($A98,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!P:P,MATCH($A98,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>4</v>
       </c>
       <c r="E98">
@@ -49735,7 +49665,7 @@
         <v>23</v>
       </c>
       <c r="D99">
-        <f>INDEX('סקרים לפי ערוץ'!R:R,MATCH($A99,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!Q:Q,MATCH($A99,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>5</v>
       </c>
       <c r="E99">
@@ -49878,9 +49808,9 @@
       <c r="C103" t="s">
         <v>13</v>
       </c>
-      <c r="D103">
-        <f>INDEX('סקרים לפי ערוץ'!H:H,MATCH($A103,'סקרים לפי ערוץ'!$A:$A,0))</f>
-        <v>0</v>
+      <c r="D103" t="e">
+        <f>INDEX('סקרים לפי ערוץ'!#REF!,MATCH($A103,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>#REF!</v>
       </c>
       <c r="E103">
         <f>COUNTIFS('מועמדים 2026'!$A:$A,$C103,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D103)</f>
@@ -49890,17 +49820,17 @@
         <f>COUNTIFS('מועמדים 2026'!$A:$A,$C103,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D103)</f>
         <v>0</v>
       </c>
-      <c r="G103">
+      <c r="G103" t="e">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>#REF!</v>
       </c>
       <c r="H103">
         <f>COUNTIFS('מועמדים 2026'!$A:$A,$C103)</f>
         <v>5</v>
       </c>
-      <c r="I103" t="str">
+      <c r="I103" t="e">
         <f t="shared" si="4"/>
-        <v/>
+        <v>#REF!</v>
       </c>
     </row>
     <row r="104" spans="1:9">
@@ -49915,7 +49845,7 @@
         <v>14</v>
       </c>
       <c r="D104">
-        <f>INDEX('סקרים לפי ערוץ'!I:I,MATCH($A104,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!H:H,MATCH($A104,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>8</v>
       </c>
       <c r="E104">
@@ -49951,7 +49881,7 @@
         <v>15</v>
       </c>
       <c r="D105">
-        <f>INDEX('סקרים לפי ערוץ'!J:J,MATCH($A105,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!I:I,MATCH($A105,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>9</v>
       </c>
       <c r="E105">
@@ -49987,7 +49917,7 @@
         <v>16</v>
       </c>
       <c r="D106">
-        <f>INDEX('סקרים לפי ערוץ'!K:K,MATCH($A106,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!J:J,MATCH($A106,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>9</v>
       </c>
       <c r="E106">
@@ -50023,7 +49953,7 @@
         <v>17</v>
       </c>
       <c r="D107">
-        <f>INDEX('סקרים לפי ערוץ'!L:L,MATCH($A107,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!K:K,MATCH($A107,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>6</v>
       </c>
       <c r="E107">
@@ -50059,7 +49989,7 @@
         <v>18</v>
       </c>
       <c r="D108">
-        <f>INDEX('סקרים לפי ערוץ'!M:M,MATCH($A108,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!L:L,MATCH($A108,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>5</v>
       </c>
       <c r="E108">
@@ -50095,7 +50025,7 @@
         <v>19</v>
       </c>
       <c r="D109">
-        <f>INDEX('סקרים לפי ערוץ'!N:N,MATCH($A109,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!M:M,MATCH($A109,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>8</v>
       </c>
       <c r="E109">
@@ -50131,7 +50061,7 @@
         <v>20</v>
       </c>
       <c r="D110">
-        <f>INDEX('סקרים לפי ערוץ'!O:O,MATCH($A110,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!N:N,MATCH($A110,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>13</v>
       </c>
       <c r="E110">
@@ -50167,7 +50097,7 @@
         <v>21</v>
       </c>
       <c r="D111">
-        <f>INDEX('סקרים לפי ערוץ'!P:P,MATCH($A111,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!O:O,MATCH($A111,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>23</v>
       </c>
       <c r="E111">
@@ -50203,7 +50133,7 @@
         <v>22</v>
       </c>
       <c r="D112">
-        <f>INDEX('סקרים לפי ערוץ'!Q:Q,MATCH($A112,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!P:P,MATCH($A112,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>0</v>
       </c>
       <c r="E112">
@@ -50239,7 +50169,7 @@
         <v>23</v>
       </c>
       <c r="D113">
-        <f>INDEX('סקרים לפי ערוץ'!R:R,MATCH($A113,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!Q:Q,MATCH($A113,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>4</v>
       </c>
       <c r="E113">
@@ -50382,9 +50312,9 @@
       <c r="C117" t="s">
         <v>13</v>
       </c>
-      <c r="D117">
-        <f>INDEX('סקרים לפי ערוץ'!H:H,MATCH($A117,'סקרים לפי ערוץ'!$A:$A,0))</f>
-        <v>0</v>
+      <c r="D117" t="e">
+        <f>INDEX('סקרים לפי ערוץ'!#REF!,MATCH($A117,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>#REF!</v>
       </c>
       <c r="E117">
         <f>COUNTIFS('מועמדים 2026'!$A:$A,$C117,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D117)</f>
@@ -50394,17 +50324,17 @@
         <f>COUNTIFS('מועמדים 2026'!$A:$A,$C117,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D117)</f>
         <v>0</v>
       </c>
-      <c r="G117">
+      <c r="G117" t="e">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>#REF!</v>
       </c>
       <c r="H117">
         <f>COUNTIFS('מועמדים 2026'!$A:$A,$C117)</f>
         <v>5</v>
       </c>
-      <c r="I117" t="str">
+      <c r="I117" t="e">
         <f t="shared" si="4"/>
-        <v/>
+        <v>#REF!</v>
       </c>
     </row>
     <row r="118" spans="1:9">
@@ -50419,7 +50349,7 @@
         <v>14</v>
       </c>
       <c r="D118">
-        <f>INDEX('סקרים לפי ערוץ'!I:I,MATCH($A118,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!H:H,MATCH($A118,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>8</v>
       </c>
       <c r="E118">
@@ -50455,7 +50385,7 @@
         <v>15</v>
       </c>
       <c r="D119">
-        <f>INDEX('סקרים לפי ערוץ'!J:J,MATCH($A119,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!I:I,MATCH($A119,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>9</v>
       </c>
       <c r="E119">
@@ -50491,7 +50421,7 @@
         <v>16</v>
       </c>
       <c r="D120">
-        <f>INDEX('סקרים לפי ערוץ'!K:K,MATCH($A120,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!J:J,MATCH($A120,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>10</v>
       </c>
       <c r="E120">
@@ -50527,7 +50457,7 @@
         <v>17</v>
       </c>
       <c r="D121">
-        <f>INDEX('סקרים לפי ערוץ'!L:L,MATCH($A121,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!K:K,MATCH($A121,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>6</v>
       </c>
       <c r="E121">
@@ -50563,7 +50493,7 @@
         <v>18</v>
       </c>
       <c r="D122">
-        <f>INDEX('סקרים לפי ערוץ'!M:M,MATCH($A122,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!L:L,MATCH($A122,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>5</v>
       </c>
       <c r="E122">
@@ -50599,7 +50529,7 @@
         <v>19</v>
       </c>
       <c r="D123">
-        <f>INDEX('סקרים לפי ערוץ'!N:N,MATCH($A123,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!M:M,MATCH($A123,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>8</v>
       </c>
       <c r="E123">
@@ -50635,7 +50565,7 @@
         <v>20</v>
       </c>
       <c r="D124">
-        <f>INDEX('סקרים לפי ערוץ'!O:O,MATCH($A124,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!N:N,MATCH($A124,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>13</v>
       </c>
       <c r="E124">
@@ -50671,7 +50601,7 @@
         <v>21</v>
       </c>
       <c r="D125">
-        <f>INDEX('סקרים לפי ערוץ'!P:P,MATCH($A125,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!O:O,MATCH($A125,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>22</v>
       </c>
       <c r="E125">
@@ -50707,7 +50637,7 @@
         <v>22</v>
       </c>
       <c r="D126">
-        <f>INDEX('סקרים לפי ערוץ'!Q:Q,MATCH($A126,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!P:P,MATCH($A126,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>0</v>
       </c>
       <c r="E126">
@@ -50743,7 +50673,7 @@
         <v>23</v>
       </c>
       <c r="D127">
-        <f>INDEX('סקרים לפי ערוץ'!R:R,MATCH($A127,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!Q:Q,MATCH($A127,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>4</v>
       </c>
       <c r="E127">
@@ -50886,9 +50816,9 @@
       <c r="C131" t="s">
         <v>13</v>
       </c>
-      <c r="D131">
-        <f>INDEX('סקרים לפי ערוץ'!H:H,MATCH($A131,'סקרים לפי ערוץ'!$A:$A,0))</f>
-        <v>0</v>
+      <c r="D131" t="e">
+        <f>INDEX('סקרים לפי ערוץ'!#REF!,MATCH($A131,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>#REF!</v>
       </c>
       <c r="E131">
         <f>COUNTIFS('מועמדים 2026'!$A:$A,$C131,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D131)</f>
@@ -50898,17 +50828,17 @@
         <f>COUNTIFS('מועמדים 2026'!$A:$A,$C131,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D131)</f>
         <v>0</v>
       </c>
-      <c r="G131">
+      <c r="G131" t="e">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>#REF!</v>
       </c>
       <c r="H131">
         <f>COUNTIFS('מועמדים 2026'!$A:$A,$C131)</f>
         <v>5</v>
       </c>
-      <c r="I131" t="str">
+      <c r="I131" t="e">
         <f t="shared" ref="I131:I141" si="7">IF(AND($D131&gt;0,$H131=0),"אין נתוני מועמדים לחישוב",IF(D131&gt;H131,"חסרים מועמדים ברשימה",""))</f>
-        <v/>
+        <v>#REF!</v>
       </c>
     </row>
     <row r="132" spans="1:9">
@@ -50923,7 +50853,7 @@
         <v>14</v>
       </c>
       <c r="D132">
-        <f>INDEX('סקרים לפי ערוץ'!I:I,MATCH($A132,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!H:H,MATCH($A132,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>7</v>
       </c>
       <c r="E132">
@@ -50959,7 +50889,7 @@
         <v>15</v>
       </c>
       <c r="D133">
-        <f>INDEX('סקרים לפי ערוץ'!J:J,MATCH($A133,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!I:I,MATCH($A133,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>7</v>
       </c>
       <c r="E133">
@@ -50995,7 +50925,7 @@
         <v>16</v>
       </c>
       <c r="D134">
-        <f>INDEX('סקרים לפי ערוץ'!K:K,MATCH($A134,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!J:J,MATCH($A134,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>10</v>
       </c>
       <c r="E134">
@@ -51031,7 +50961,7 @@
         <v>17</v>
       </c>
       <c r="D135">
-        <f>INDEX('סקרים לפי ערוץ'!L:L,MATCH($A135,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!K:K,MATCH($A135,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>6</v>
       </c>
       <c r="E135">
@@ -51067,7 +50997,7 @@
         <v>18</v>
       </c>
       <c r="D136">
-        <f>INDEX('סקרים לפי ערוץ'!M:M,MATCH($A136,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!L:L,MATCH($A136,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>5</v>
       </c>
       <c r="E136">
@@ -51103,7 +51033,7 @@
         <v>19</v>
       </c>
       <c r="D137">
-        <f>INDEX('סקרים לפי ערוץ'!N:N,MATCH($A137,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!M:M,MATCH($A137,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>9</v>
       </c>
       <c r="E137">
@@ -51139,7 +51069,7 @@
         <v>20</v>
       </c>
       <c r="D138">
-        <f>INDEX('סקרים לפי ערוץ'!O:O,MATCH($A138,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!N:N,MATCH($A138,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>11</v>
       </c>
       <c r="E138">
@@ -51175,7 +51105,7 @@
         <v>21</v>
       </c>
       <c r="D139">
-        <f>INDEX('סקרים לפי ערוץ'!P:P,MATCH($A139,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!O:O,MATCH($A139,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>20</v>
       </c>
       <c r="E139">
@@ -51211,7 +51141,7 @@
         <v>22</v>
       </c>
       <c r="D140">
-        <f>INDEX('סקרים לפי ערוץ'!Q:Q,MATCH($A140,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!P:P,MATCH($A140,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>4</v>
       </c>
       <c r="E140">
@@ -51247,7 +51177,7 @@
         <v>23</v>
       </c>
       <c r="D141">
-        <f>INDEX('סקרים לפי ערוץ'!R:R,MATCH($A141,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <f>INDEX('סקרים לפי ערוץ'!Q:Q,MATCH($A141,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>0</v>
       </c>
       <c r="E141">

</xml_diff>